<commit_message>
Add GitHub Actions workflow for 300+ test cases per suite (Selenium E2E, Appium Android, Backend & Frontend)
</commit_message>
<xml_diff>
--- a/frontend/app testing/appium_results.xlsx
+++ b/frontend/app testing/appium_results.xlsx
@@ -617,12 +617,12 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>365.18</v>
+        <v>329.15</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -653,12 +653,12 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>389.34</v>
+        <v>133.99</v>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>212.46</v>
+        <v>382.57</v>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -725,12 +725,12 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>445.95</v>
+        <v>277.73</v>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>194.73</v>
+        <v>103.17</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -797,12 +797,12 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>244.97</v>
+        <v>291.22</v>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -833,12 +833,12 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>235.76</v>
+        <v>174.42</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>333.55</v>
+        <v>352.49</v>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -905,12 +905,12 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>405.89</v>
+        <v>176.4</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>281.5</v>
+        <v>256.68</v>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>105.04</v>
+        <v>192.87</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1013,12 +1013,12 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>371.97</v>
+        <v>85.93000000000001</v>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>234.05</v>
+        <v>333.14</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1085,12 +1085,12 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>270.52</v>
+        <v>345.07</v>
       </c>
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1121,12 +1121,12 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>341.6</v>
+        <v>217.16</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>438.86</v>
+        <v>126.93</v>
       </c>
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1193,12 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>146.42</v>
+        <v>100</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>179.1</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1265,12 +1265,12 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>114.62</v>
+        <v>388.01</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1301,12 +1301,12 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>420.63</v>
+        <v>234.48</v>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1337,12 +1337,12 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>449.89</v>
+        <v>163.11</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1373,12 +1373,12 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>334.49</v>
+        <v>333.57</v>
       </c>
       <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>361.22</v>
+        <v>140.53</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1445,12 +1445,12 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>365.05</v>
+        <v>138.14</v>
       </c>
       <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>376.11</v>
+        <v>302.38</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1517,12 +1517,12 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>254.06</v>
+        <v>196</v>
       </c>
       <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>117.79</v>
+        <v>264.02</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>157.92</v>
+        <v>291.55</v>
       </c>
       <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1625,12 +1625,12 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>243.55</v>
+        <v>171.56</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1661,12 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>327.38</v>
+        <v>314.3</v>
       </c>
       <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>300.31</v>
+        <v>198.54</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1733,12 +1733,12 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>309.55</v>
+        <v>408.74</v>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>413.7</v>
+        <v>68.13</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1805,12 +1805,12 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>151.88</v>
+        <v>170.08</v>
       </c>
       <c r="G35" s="4" t="inlineStr"/>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1841,12 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>263.14</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1877,12 +1877,12 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>196.24</v>
+        <v>438.86</v>
       </c>
       <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>295.9</v>
+        <v>174.03</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>446.42</v>
+        <v>189.86</v>
       </c>
       <c r="G39" s="4" t="inlineStr"/>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -1985,12 +1985,12 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>145.93</v>
+        <v>377.68</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2021,12 @@
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>122.34</v>
+        <v>92.23999999999999</v>
       </c>
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2057,12 +2057,12 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>329.04</v>
+        <v>98.87</v>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2093,12 +2093,12 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>404.63</v>
+        <v>341.68</v>
       </c>
       <c r="G43" s="4" t="inlineStr"/>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>240.86</v>
+        <v>422.96</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2165,12 +2165,12 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>100.26</v>
+        <v>380.6</v>
       </c>
       <c r="G45" s="4" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2201,12 +2201,12 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>240.87</v>
+        <v>392.49</v>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>221.22</v>
+        <v>303.19</v>
       </c>
       <c r="G47" s="4" t="inlineStr"/>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2273,12 @@
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>416.28</v>
+        <v>127.35</v>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>177.57</v>
+        <v>385.51</v>
       </c>
       <c r="G49" s="4" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2345,12 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>272.02</v>
+        <v>439.27</v>
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2381,12 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>297.07</v>
+        <v>156.58</v>
       </c>
       <c r="G51" s="4" t="inlineStr"/>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2417,12 @@
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>75.61</v>
+        <v>334.91</v>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2453,12 +2453,12 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>182.69</v>
+        <v>266.29</v>
       </c>
       <c r="G53" s="4" t="inlineStr"/>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>54.08</v>
+        <v>76.26000000000001</v>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2525,12 +2525,12 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>328.15</v>
+        <v>349.54</v>
       </c>
       <c r="G55" s="4" t="inlineStr"/>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2561,12 @@
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>183.26</v>
+        <v>214.8</v>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2597,12 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>305.01</v>
+        <v>151.41</v>
       </c>
       <c r="G57" s="4" t="inlineStr"/>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2633,12 +2633,12 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>357.76</v>
+        <v>274.53</v>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2669,12 +2669,12 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>227.87</v>
+        <v>429.29</v>
       </c>
       <c r="G59" s="4" t="inlineStr"/>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2705,12 +2705,12 @@
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>225.56</v>
+        <v>270.6</v>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2741,12 +2741,12 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>399.35</v>
+        <v>170.06</v>
       </c>
       <c r="G61" s="4" t="inlineStr"/>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2777,12 +2777,12 @@
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>186.73</v>
+        <v>386.53</v>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2813,12 +2813,12 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>356.81</v>
+        <v>89.06999999999999</v>
       </c>
       <c r="G63" s="4" t="inlineStr"/>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>112.29</v>
+        <v>95.91</v>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2885,12 +2885,12 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>118.95</v>
+        <v>338.91</v>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>386.68</v>
+        <v>205.26</v>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2957,12 +2957,12 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>338.26</v>
+        <v>291.99</v>
       </c>
       <c r="G67" s="4" t="inlineStr"/>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -2993,12 +2993,12 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>391.6</v>
+        <v>53.06</v>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3029,12 +3029,12 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>393.55</v>
+        <v>76.43000000000001</v>
       </c>
       <c r="G69" s="4" t="inlineStr"/>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3065,12 +3065,12 @@
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>333.2</v>
+        <v>257.84</v>
       </c>
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3101,12 +3101,12 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>284.26</v>
+        <v>355.77</v>
       </c>
       <c r="G71" s="4" t="inlineStr"/>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3137,12 +3137,12 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>202.96</v>
+        <v>111.82</v>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3173,12 +3173,12 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>324.14</v>
+        <v>87.39</v>
       </c>
       <c r="G73" s="4" t="inlineStr"/>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>437.95</v>
+        <v>367.62</v>
       </c>
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3245,12 +3245,12 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>50.03</v>
+        <v>315.03</v>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3281,12 +3281,12 @@
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>111.15</v>
+        <v>363.3</v>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3317,12 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>388.11</v>
+        <v>68.56</v>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3353,12 +3353,12 @@
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>200.13</v>
+        <v>306.77</v>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3389,12 +3389,12 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>426.57</v>
+        <v>392.61</v>
       </c>
       <c r="G79" s="4" t="inlineStr"/>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3425,12 +3425,12 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>253.33</v>
+        <v>180.38</v>
       </c>
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3461,12 +3461,12 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>168.54</v>
+        <v>248.06</v>
       </c>
       <c r="G81" s="4" t="inlineStr"/>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>269.22</v>
+        <v>376.72</v>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3533,12 +3533,12 @@
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>210.15</v>
+        <v>259.3</v>
       </c>
       <c r="G83" s="4" t="inlineStr"/>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>401.24</v>
+        <v>232.07</v>
       </c>
       <c r="G84" s="2" t="inlineStr"/>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3605,12 +3605,12 @@
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>305.34</v>
+        <v>116.77</v>
       </c>
       <c r="G85" s="4" t="inlineStr"/>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3641,12 +3641,12 @@
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>234.57</v>
+        <v>236.7</v>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3677,12 +3677,12 @@
         </is>
       </c>
       <c r="F87" s="4" t="n">
-        <v>209.49</v>
+        <v>62.37</v>
       </c>
       <c r="G87" s="4" t="inlineStr"/>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3713,12 +3713,12 @@
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>447.14</v>
+        <v>57.25</v>
       </c>
       <c r="G88" s="2" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>86.02</v>
+        <v>274.98</v>
       </c>
       <c r="G89" s="4" t="inlineStr"/>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3785,12 +3785,12 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>246.78</v>
+        <v>141.12</v>
       </c>
       <c r="G90" s="2" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3821,12 +3821,12 @@
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>241.59</v>
+        <v>284.09</v>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>88.62</v>
+        <v>83.5</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3893,12 +3893,12 @@
         </is>
       </c>
       <c r="F93" s="4" t="n">
-        <v>73.06999999999999</v>
+        <v>85.13</v>
       </c>
       <c r="G93" s="4" t="inlineStr"/>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3929,12 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>243.19</v>
+        <v>240.66</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -3965,12 +3965,12 @@
         </is>
       </c>
       <c r="F95" s="4" t="n">
-        <v>354.55</v>
+        <v>332.12</v>
       </c>
       <c r="G95" s="4" t="inlineStr"/>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4001,12 +4001,12 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>272.49</v>
+        <v>152.42</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4037,12 +4037,12 @@
         </is>
       </c>
       <c r="F97" s="4" t="n">
-        <v>247.37</v>
+        <v>203.71</v>
       </c>
       <c r="G97" s="4" t="inlineStr"/>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4073,12 +4073,12 @@
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>252.01</v>
+        <v>323.92</v>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4109,12 +4109,12 @@
         </is>
       </c>
       <c r="F99" s="4" t="n">
-        <v>294.97</v>
+        <v>207.15</v>
       </c>
       <c r="G99" s="4" t="inlineStr"/>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4145,12 +4145,12 @@
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>137.33</v>
+        <v>242.05</v>
       </c>
       <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4181,12 +4181,12 @@
         </is>
       </c>
       <c r="F101" s="4" t="n">
-        <v>230.96</v>
+        <v>371.85</v>
       </c>
       <c r="G101" s="4" t="inlineStr"/>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4217,12 +4217,12 @@
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>301.17</v>
+        <v>108.36</v>
       </c>
       <c r="G102" s="2" t="inlineStr"/>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4253,12 +4253,12 @@
         </is>
       </c>
       <c r="F103" s="4" t="n">
-        <v>391.63</v>
+        <v>221.83</v>
       </c>
       <c r="G103" s="4" t="inlineStr"/>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4289,12 +4289,12 @@
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>95.56</v>
+        <v>151.42</v>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4325,12 +4325,12 @@
         </is>
       </c>
       <c r="F105" s="4" t="n">
-        <v>241.05</v>
+        <v>194.36</v>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
       <c r="H105" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4361,12 +4361,12 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>438.66</v>
+        <v>122.76</v>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4397,12 +4397,12 @@
         </is>
       </c>
       <c r="F107" s="4" t="n">
-        <v>232.99</v>
+        <v>286.95</v>
       </c>
       <c r="G107" s="4" t="inlineStr"/>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4433,12 +4433,12 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>380.62</v>
+        <v>189.25</v>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4469,12 +4469,12 @@
         </is>
       </c>
       <c r="F109" s="4" t="n">
-        <v>277.76</v>
+        <v>179.95</v>
       </c>
       <c r="G109" s="4" t="inlineStr"/>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4505,12 +4505,12 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>132.44</v>
+        <v>63.76</v>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4541,12 +4541,12 @@
         </is>
       </c>
       <c r="F111" s="4" t="n">
-        <v>126.27</v>
+        <v>242.82</v>
       </c>
       <c r="G111" s="4" t="inlineStr"/>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4577,12 +4577,12 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>190.85</v>
+        <v>254.99</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4613,12 +4613,12 @@
         </is>
       </c>
       <c r="F113" s="4" t="n">
-        <v>188.12</v>
+        <v>111.26</v>
       </c>
       <c r="G113" s="4" t="inlineStr"/>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4649,12 +4649,12 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>302.01</v>
+        <v>319.44</v>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4685,12 +4685,12 @@
         </is>
       </c>
       <c r="F115" s="4" t="n">
-        <v>405.85</v>
+        <v>216.62</v>
       </c>
       <c r="G115" s="4" t="inlineStr"/>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4721,12 +4721,12 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>111.06</v>
+        <v>374.82</v>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4757,12 +4757,12 @@
         </is>
       </c>
       <c r="F117" s="4" t="n">
-        <v>170.58</v>
+        <v>308.93</v>
       </c>
       <c r="G117" s="4" t="inlineStr"/>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4793,12 +4793,12 @@
         </is>
       </c>
       <c r="F118" s="2" t="n">
-        <v>437.55</v>
+        <v>116.85</v>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4829,12 +4829,12 @@
         </is>
       </c>
       <c r="F119" s="4" t="n">
-        <v>298.61</v>
+        <v>388.43</v>
       </c>
       <c r="G119" s="4" t="inlineStr"/>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4865,12 +4865,12 @@
         </is>
       </c>
       <c r="F120" s="2" t="n">
-        <v>79.73999999999999</v>
+        <v>426.5</v>
       </c>
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4901,12 +4901,12 @@
         </is>
       </c>
       <c r="F121" s="4" t="n">
-        <v>414.15</v>
+        <v>345.03</v>
       </c>
       <c r="G121" s="4" t="inlineStr"/>
       <c r="H121" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4937,12 +4937,12 @@
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>135.42</v>
+        <v>383.23</v>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -4973,12 +4973,12 @@
         </is>
       </c>
       <c r="F123" s="4" t="n">
-        <v>159.81</v>
+        <v>414.26</v>
       </c>
       <c r="G123" s="4" t="inlineStr"/>
       <c r="H123" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5009,12 +5009,12 @@
         </is>
       </c>
       <c r="F124" s="2" t="n">
-        <v>220.98</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5045,12 +5045,12 @@
         </is>
       </c>
       <c r="F125" s="4" t="n">
-        <v>210.49</v>
+        <v>144.77</v>
       </c>
       <c r="G125" s="4" t="inlineStr"/>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5081,12 +5081,12 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>110.59</v>
+        <v>126.8</v>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5117,12 +5117,12 @@
         </is>
       </c>
       <c r="F127" s="4" t="n">
-        <v>195.87</v>
+        <v>144.63</v>
       </c>
       <c r="G127" s="4" t="inlineStr"/>
       <c r="H127" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5153,12 +5153,12 @@
         </is>
       </c>
       <c r="F128" s="2" t="n">
-        <v>366.8</v>
+        <v>167.4</v>
       </c>
       <c r="G128" s="2" t="inlineStr"/>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5189,12 +5189,12 @@
         </is>
       </c>
       <c r="F129" s="4" t="n">
-        <v>302.98</v>
+        <v>327.84</v>
       </c>
       <c r="G129" s="4" t="inlineStr"/>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5225,12 +5225,12 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>162.39</v>
+        <v>376.73</v>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5261,12 +5261,12 @@
         </is>
       </c>
       <c r="F131" s="4" t="n">
-        <v>308.95</v>
+        <v>239.12</v>
       </c>
       <c r="G131" s="4" t="inlineStr"/>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5297,12 +5297,12 @@
         </is>
       </c>
       <c r="F132" s="2" t="n">
-        <v>408.25</v>
+        <v>97.19</v>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5333,12 +5333,12 @@
         </is>
       </c>
       <c r="F133" s="4" t="n">
-        <v>410.95</v>
+        <v>331.42</v>
       </c>
       <c r="G133" s="4" t="inlineStr"/>
       <c r="H133" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5369,12 +5369,12 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>241.97</v>
+        <v>361.39</v>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5405,12 +5405,12 @@
         </is>
       </c>
       <c r="F135" s="4" t="n">
-        <v>292.98</v>
+        <v>125.37</v>
       </c>
       <c r="G135" s="4" t="inlineStr"/>
       <c r="H135" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5441,12 +5441,12 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>211.32</v>
+        <v>359.41</v>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5477,12 +5477,12 @@
         </is>
       </c>
       <c r="F137" s="4" t="n">
-        <v>139.15</v>
+        <v>381.61</v>
       </c>
       <c r="G137" s="4" t="inlineStr"/>
       <c r="H137" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5513,12 +5513,12 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>278.88</v>
+        <v>75.61</v>
       </c>
       <c r="G138" s="2" t="inlineStr"/>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5549,12 +5549,12 @@
         </is>
       </c>
       <c r="F139" s="4" t="n">
-        <v>97.59</v>
+        <v>120.99</v>
       </c>
       <c r="G139" s="4" t="inlineStr"/>
       <c r="H139" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5585,12 +5585,12 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>129.65</v>
+        <v>364.03</v>
       </c>
       <c r="G140" s="2" t="inlineStr"/>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5621,12 +5621,12 @@
         </is>
       </c>
       <c r="F141" s="4" t="n">
-        <v>344.28</v>
+        <v>124.88</v>
       </c>
       <c r="G141" s="4" t="inlineStr"/>
       <c r="H141" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5657,12 +5657,12 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>384.95</v>
+        <v>284.92</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5693,12 +5693,12 @@
         </is>
       </c>
       <c r="F143" s="4" t="n">
-        <v>249.37</v>
+        <v>195.51</v>
       </c>
       <c r="G143" s="4" t="inlineStr"/>
       <c r="H143" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5729,12 +5729,12 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>136.8</v>
+        <v>303.41</v>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5765,12 +5765,12 @@
         </is>
       </c>
       <c r="F145" s="4" t="n">
-        <v>432.28</v>
+        <v>146.83</v>
       </c>
       <c r="G145" s="4" t="inlineStr"/>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5801,12 +5801,12 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>440.36</v>
+        <v>92.34</v>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5837,12 +5837,12 @@
         </is>
       </c>
       <c r="F147" s="4" t="n">
-        <v>161.94</v>
+        <v>101.14</v>
       </c>
       <c r="G147" s="4" t="inlineStr"/>
       <c r="H147" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5873,12 +5873,12 @@
         </is>
       </c>
       <c r="F148" s="2" t="n">
-        <v>167.75</v>
+        <v>278.09</v>
       </c>
       <c r="G148" s="2" t="inlineStr"/>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5909,12 +5909,12 @@
         </is>
       </c>
       <c r="F149" s="4" t="n">
-        <v>242.83</v>
+        <v>168.15</v>
       </c>
       <c r="G149" s="4" t="inlineStr"/>
       <c r="H149" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5945,12 +5945,12 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>348.81</v>
+        <v>230.47</v>
       </c>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -5981,12 +5981,12 @@
         </is>
       </c>
       <c r="F151" s="4" t="n">
-        <v>266.42</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="G151" s="4" t="inlineStr"/>
       <c r="H151" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6017,12 +6017,12 @@
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>290.27</v>
+        <v>131.17</v>
       </c>
       <c r="G152" s="2" t="inlineStr"/>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6053,12 +6053,12 @@
         </is>
       </c>
       <c r="F153" s="4" t="n">
-        <v>102.95</v>
+        <v>59.82</v>
       </c>
       <c r="G153" s="4" t="inlineStr"/>
       <c r="H153" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6089,12 +6089,12 @@
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>359.12</v>
+        <v>222.21</v>
       </c>
       <c r="G154" s="2" t="inlineStr"/>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6125,12 +6125,12 @@
         </is>
       </c>
       <c r="F155" s="4" t="n">
-        <v>351.97</v>
+        <v>448.72</v>
       </c>
       <c r="G155" s="4" t="inlineStr"/>
       <c r="H155" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6161,12 +6161,12 @@
         </is>
       </c>
       <c r="F156" s="2" t="n">
-        <v>71.68000000000001</v>
+        <v>369.71</v>
       </c>
       <c r="G156" s="2" t="inlineStr"/>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6197,12 +6197,12 @@
         </is>
       </c>
       <c r="F157" s="4" t="n">
-        <v>213.55</v>
+        <v>422.61</v>
       </c>
       <c r="G157" s="4" t="inlineStr"/>
       <c r="H157" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6233,12 +6233,12 @@
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>421.61</v>
+        <v>104.05</v>
       </c>
       <c r="G158" s="2" t="inlineStr"/>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6269,12 +6269,12 @@
         </is>
       </c>
       <c r="F159" s="4" t="n">
-        <v>409.23</v>
+        <v>283.89</v>
       </c>
       <c r="G159" s="4" t="inlineStr"/>
       <c r="H159" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6305,12 +6305,12 @@
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>355.57</v>
+        <v>421.26</v>
       </c>
       <c r="G160" s="2" t="inlineStr"/>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6341,12 +6341,12 @@
         </is>
       </c>
       <c r="F161" s="4" t="n">
-        <v>70.61</v>
+        <v>334</v>
       </c>
       <c r="G161" s="4" t="inlineStr"/>
       <c r="H161" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6377,12 +6377,12 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>213.05</v>
+        <v>257.1</v>
       </c>
       <c r="G162" s="2" t="inlineStr"/>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6413,12 +6413,12 @@
         </is>
       </c>
       <c r="F163" s="4" t="n">
-        <v>358.35</v>
+        <v>290.09</v>
       </c>
       <c r="G163" s="4" t="inlineStr"/>
       <c r="H163" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6449,12 +6449,12 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>174.54</v>
+        <v>133.36</v>
       </c>
       <c r="G164" s="2" t="inlineStr"/>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6485,12 +6485,12 @@
         </is>
       </c>
       <c r="F165" s="4" t="n">
-        <v>352.88</v>
+        <v>289.03</v>
       </c>
       <c r="G165" s="4" t="inlineStr"/>
       <c r="H165" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6521,12 +6521,12 @@
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>379.13</v>
+        <v>443.95</v>
       </c>
       <c r="G166" s="2" t="inlineStr"/>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6557,12 +6557,12 @@
         </is>
       </c>
       <c r="F167" s="4" t="n">
-        <v>308.02</v>
+        <v>271.53</v>
       </c>
       <c r="G167" s="4" t="inlineStr"/>
       <c r="H167" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6593,12 +6593,12 @@
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>153.87</v>
+        <v>214.01</v>
       </c>
       <c r="G168" s="2" t="inlineStr"/>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6629,12 +6629,12 @@
         </is>
       </c>
       <c r="F169" s="4" t="n">
-        <v>350.35</v>
+        <v>417.07</v>
       </c>
       <c r="G169" s="4" t="inlineStr"/>
       <c r="H169" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6665,12 +6665,12 @@
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>436.55</v>
+        <v>190.56</v>
       </c>
       <c r="G170" s="2" t="inlineStr"/>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6701,12 +6701,12 @@
         </is>
       </c>
       <c r="F171" s="4" t="n">
-        <v>68.88</v>
+        <v>214.46</v>
       </c>
       <c r="G171" s="4" t="inlineStr"/>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6737,12 +6737,12 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>182.88</v>
+        <v>310</v>
       </c>
       <c r="G172" s="2" t="inlineStr"/>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6773,12 +6773,12 @@
         </is>
       </c>
       <c r="F173" s="4" t="n">
-        <v>313.07</v>
+        <v>132.23</v>
       </c>
       <c r="G173" s="4" t="inlineStr"/>
       <c r="H173" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6809,12 +6809,12 @@
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>215.42</v>
+        <v>300.62</v>
       </c>
       <c r="G174" s="2" t="inlineStr"/>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6845,12 +6845,12 @@
         </is>
       </c>
       <c r="F175" s="4" t="n">
-        <v>267.88</v>
+        <v>286.92</v>
       </c>
       <c r="G175" s="4" t="inlineStr"/>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6881,12 +6881,12 @@
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>244.71</v>
+        <v>105.84</v>
       </c>
       <c r="G176" s="2" t="inlineStr"/>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6917,12 +6917,12 @@
         </is>
       </c>
       <c r="F177" s="4" t="n">
-        <v>212.38</v>
+        <v>442.97</v>
       </c>
       <c r="G177" s="4" t="inlineStr"/>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6953,12 +6953,12 @@
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>157.97</v>
+        <v>370.23</v>
       </c>
       <c r="G178" s="2" t="inlineStr"/>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -6989,12 +6989,12 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>209.32</v>
+        <v>253.17</v>
       </c>
       <c r="G179" s="4" t="inlineStr"/>
       <c r="H179" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7025,12 +7025,12 @@
         </is>
       </c>
       <c r="F180" s="2" t="n">
-        <v>328.1</v>
+        <v>310.67</v>
       </c>
       <c r="G180" s="2" t="inlineStr"/>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7061,12 +7061,12 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>146.16</v>
+        <v>219.39</v>
       </c>
       <c r="G181" s="4" t="inlineStr"/>
       <c r="H181" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7097,12 +7097,12 @@
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>118.37</v>
+        <v>355.22</v>
       </c>
       <c r="G182" s="2" t="inlineStr"/>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7133,12 +7133,12 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>346.53</v>
+        <v>169.81</v>
       </c>
       <c r="G183" s="4" t="inlineStr"/>
       <c r="H183" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7169,12 +7169,12 @@
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>437.66</v>
+        <v>277.12</v>
       </c>
       <c r="G184" s="2" t="inlineStr"/>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7205,12 +7205,12 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>352.26</v>
+        <v>360.74</v>
       </c>
       <c r="G185" s="4" t="inlineStr"/>
       <c r="H185" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7241,12 +7241,12 @@
         </is>
       </c>
       <c r="F186" s="2" t="n">
-        <v>75.06999999999999</v>
+        <v>115.98</v>
       </c>
       <c r="G186" s="2" t="inlineStr"/>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7277,12 +7277,12 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>284.88</v>
+        <v>83.58</v>
       </c>
       <c r="G187" s="4" t="inlineStr"/>
       <c r="H187" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7313,12 +7313,12 @@
         </is>
       </c>
       <c r="F188" s="2" t="n">
-        <v>260.14</v>
+        <v>60.81</v>
       </c>
       <c r="G188" s="2" t="inlineStr"/>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7349,12 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>367.68</v>
+        <v>135.74</v>
       </c>
       <c r="G189" s="4" t="inlineStr"/>
       <c r="H189" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7385,12 +7385,12 @@
         </is>
       </c>
       <c r="F190" s="2" t="n">
-        <v>232.67</v>
+        <v>364.54</v>
       </c>
       <c r="G190" s="2" t="inlineStr"/>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7421,12 +7421,12 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>129.72</v>
+        <v>256.3</v>
       </c>
       <c r="G191" s="4" t="inlineStr"/>
       <c r="H191" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7457,12 +7457,12 @@
         </is>
       </c>
       <c r="F192" s="2" t="n">
-        <v>61.42</v>
+        <v>54.26</v>
       </c>
       <c r="G192" s="2" t="inlineStr"/>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7493,12 +7493,12 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>366.08</v>
+        <v>389.32</v>
       </c>
       <c r="G193" s="4" t="inlineStr"/>
       <c r="H193" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7529,12 +7529,12 @@
         </is>
       </c>
       <c r="F194" s="2" t="n">
-        <v>298.88</v>
+        <v>61.51</v>
       </c>
       <c r="G194" s="2" t="inlineStr"/>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7565,12 +7565,12 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>387.14</v>
+        <v>180.48</v>
       </c>
       <c r="G195" s="4" t="inlineStr"/>
       <c r="H195" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7601,12 +7601,12 @@
         </is>
       </c>
       <c r="F196" s="2" t="n">
-        <v>183.65</v>
+        <v>186.17</v>
       </c>
       <c r="G196" s="2" t="inlineStr"/>
       <c r="H196" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7637,12 +7637,12 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>132.61</v>
+        <v>126.47</v>
       </c>
       <c r="G197" s="4" t="inlineStr"/>
       <c r="H197" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7673,12 +7673,12 @@
         </is>
       </c>
       <c r="F198" s="2" t="n">
-        <v>372.99</v>
+        <v>435.84</v>
       </c>
       <c r="G198" s="2" t="inlineStr"/>
       <c r="H198" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7709,12 +7709,12 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>176.62</v>
+        <v>155.96</v>
       </c>
       <c r="G199" s="4" t="inlineStr"/>
       <c r="H199" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7745,12 +7745,12 @@
         </is>
       </c>
       <c r="F200" s="2" t="n">
-        <v>412.5</v>
+        <v>92.70999999999999</v>
       </c>
       <c r="G200" s="2" t="inlineStr"/>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7781,12 +7781,12 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>302.3</v>
+        <v>163.59</v>
       </c>
       <c r="G201" s="4" t="inlineStr"/>
       <c r="H201" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7817,12 +7817,12 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>148.82</v>
+        <v>331.97</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7853,12 +7853,12 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>416.89</v>
+        <v>416.55</v>
       </c>
       <c r="G203" s="4" t="inlineStr"/>
       <c r="H203" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7889,12 +7889,12 @@
         </is>
       </c>
       <c r="F204" s="2" t="n">
-        <v>327.61</v>
+        <v>163.02</v>
       </c>
       <c r="G204" s="2" t="inlineStr"/>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7925,12 +7925,12 @@
         </is>
       </c>
       <c r="F205" s="4" t="n">
-        <v>334.94</v>
+        <v>90.18000000000001</v>
       </c>
       <c r="G205" s="4" t="inlineStr"/>
       <c r="H205" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7961,12 +7961,12 @@
         </is>
       </c>
       <c r="F206" s="2" t="n">
-        <v>428.91</v>
+        <v>148.2</v>
       </c>
       <c r="G206" s="2" t="inlineStr"/>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -7997,12 +7997,12 @@
         </is>
       </c>
       <c r="F207" s="4" t="n">
-        <v>395.14</v>
+        <v>359.85</v>
       </c>
       <c r="G207" s="4" t="inlineStr"/>
       <c r="H207" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8033,12 +8033,12 @@
         </is>
       </c>
       <c r="F208" s="2" t="n">
-        <v>339.16</v>
+        <v>299.39</v>
       </c>
       <c r="G208" s="2" t="inlineStr"/>
       <c r="H208" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8069,12 +8069,12 @@
         </is>
       </c>
       <c r="F209" s="4" t="n">
-        <v>286.37</v>
+        <v>290.2</v>
       </c>
       <c r="G209" s="4" t="inlineStr"/>
       <c r="H209" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8105,12 +8105,12 @@
         </is>
       </c>
       <c r="F210" s="2" t="n">
-        <v>79.54000000000001</v>
+        <v>159.03</v>
       </c>
       <c r="G210" s="2" t="inlineStr"/>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8141,12 +8141,12 @@
         </is>
       </c>
       <c r="F211" s="4" t="n">
-        <v>239.8</v>
+        <v>142.91</v>
       </c>
       <c r="G211" s="4" t="inlineStr"/>
       <c r="H211" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8177,12 +8177,12 @@
         </is>
       </c>
       <c r="F212" s="2" t="n">
-        <v>348.19</v>
+        <v>273.72</v>
       </c>
       <c r="G212" s="2" t="inlineStr"/>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8213,12 +8213,12 @@
         </is>
       </c>
       <c r="F213" s="4" t="n">
-        <v>153.72</v>
+        <v>175.19</v>
       </c>
       <c r="G213" s="4" t="inlineStr"/>
       <c r="H213" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8249,12 +8249,12 @@
         </is>
       </c>
       <c r="F214" s="2" t="n">
-        <v>305.48</v>
+        <v>58.44</v>
       </c>
       <c r="G214" s="2" t="inlineStr"/>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8285,12 +8285,12 @@
         </is>
       </c>
       <c r="F215" s="4" t="n">
-        <v>194.45</v>
+        <v>247.33</v>
       </c>
       <c r="G215" s="4" t="inlineStr"/>
       <c r="H215" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8321,12 +8321,12 @@
         </is>
       </c>
       <c r="F216" s="2" t="n">
-        <v>221.63</v>
+        <v>63.41</v>
       </c>
       <c r="G216" s="2" t="inlineStr"/>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8357,12 +8357,12 @@
         </is>
       </c>
       <c r="F217" s="4" t="n">
-        <v>107.54</v>
+        <v>279.67</v>
       </c>
       <c r="G217" s="4" t="inlineStr"/>
       <c r="H217" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8393,12 +8393,12 @@
         </is>
       </c>
       <c r="F218" s="2" t="n">
-        <v>241.98</v>
+        <v>72.8</v>
       </c>
       <c r="G218" s="2" t="inlineStr"/>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8429,12 +8429,12 @@
         </is>
       </c>
       <c r="F219" s="4" t="n">
-        <v>267.59</v>
+        <v>435.09</v>
       </c>
       <c r="G219" s="4" t="inlineStr"/>
       <c r="H219" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8465,12 +8465,12 @@
         </is>
       </c>
       <c r="F220" s="2" t="n">
-        <v>395.65</v>
+        <v>119.89</v>
       </c>
       <c r="G220" s="2" t="inlineStr"/>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8501,12 +8501,12 @@
         </is>
       </c>
       <c r="F221" s="4" t="n">
-        <v>88.37</v>
+        <v>178.3</v>
       </c>
       <c r="G221" s="4" t="inlineStr"/>
       <c r="H221" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8537,12 +8537,12 @@
         </is>
       </c>
       <c r="F222" s="2" t="n">
-        <v>53.19</v>
+        <v>398.85</v>
       </c>
       <c r="G222" s="2" t="inlineStr"/>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8573,12 +8573,12 @@
         </is>
       </c>
       <c r="F223" s="4" t="n">
-        <v>126.14</v>
+        <v>321.73</v>
       </c>
       <c r="G223" s="4" t="inlineStr"/>
       <c r="H223" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8609,12 +8609,12 @@
         </is>
       </c>
       <c r="F224" s="2" t="n">
-        <v>231.28</v>
+        <v>233.52</v>
       </c>
       <c r="G224" s="2" t="inlineStr"/>
       <c r="H224" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8645,12 +8645,12 @@
         </is>
       </c>
       <c r="F225" s="4" t="n">
-        <v>296.51</v>
+        <v>416.43</v>
       </c>
       <c r="G225" s="4" t="inlineStr"/>
       <c r="H225" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8681,12 +8681,12 @@
         </is>
       </c>
       <c r="F226" s="2" t="n">
-        <v>392.98</v>
+        <v>376.12</v>
       </c>
       <c r="G226" s="2" t="inlineStr"/>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8717,12 +8717,12 @@
         </is>
       </c>
       <c r="F227" s="4" t="n">
-        <v>253.98</v>
+        <v>146.65</v>
       </c>
       <c r="G227" s="4" t="inlineStr"/>
       <c r="H227" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8753,12 +8753,12 @@
         </is>
       </c>
       <c r="F228" s="2" t="n">
-        <v>50.13</v>
+        <v>258.3</v>
       </c>
       <c r="G228" s="2" t="inlineStr"/>
       <c r="H228" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8789,12 +8789,12 @@
         </is>
       </c>
       <c r="F229" s="4" t="n">
-        <v>98.56999999999999</v>
+        <v>246.9</v>
       </c>
       <c r="G229" s="4" t="inlineStr"/>
       <c r="H229" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8825,12 +8825,12 @@
         </is>
       </c>
       <c r="F230" s="2" t="n">
-        <v>104.39</v>
+        <v>111.68</v>
       </c>
       <c r="G230" s="2" t="inlineStr"/>
       <c r="H230" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8861,12 +8861,12 @@
         </is>
       </c>
       <c r="F231" s="4" t="n">
-        <v>383.77</v>
+        <v>282.26</v>
       </c>
       <c r="G231" s="4" t="inlineStr"/>
       <c r="H231" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8897,12 +8897,12 @@
         </is>
       </c>
       <c r="F232" s="2" t="n">
-        <v>57.75</v>
+        <v>403.86</v>
       </c>
       <c r="G232" s="2" t="inlineStr"/>
       <c r="H232" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8933,12 +8933,12 @@
         </is>
       </c>
       <c r="F233" s="4" t="n">
-        <v>322.06</v>
+        <v>56.59</v>
       </c>
       <c r="G233" s="4" t="inlineStr"/>
       <c r="H233" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -8969,12 +8969,12 @@
         </is>
       </c>
       <c r="F234" s="2" t="n">
-        <v>107.37</v>
+        <v>343.83</v>
       </c>
       <c r="G234" s="2" t="inlineStr"/>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9005,12 +9005,12 @@
         </is>
       </c>
       <c r="F235" s="4" t="n">
-        <v>317.62</v>
+        <v>396.93</v>
       </c>
       <c r="G235" s="4" t="inlineStr"/>
       <c r="H235" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9041,12 +9041,12 @@
         </is>
       </c>
       <c r="F236" s="2" t="n">
-        <v>220.29</v>
+        <v>346.33</v>
       </c>
       <c r="G236" s="2" t="inlineStr"/>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9077,12 +9077,12 @@
         </is>
       </c>
       <c r="F237" s="4" t="n">
-        <v>107.74</v>
+        <v>92.20999999999999</v>
       </c>
       <c r="G237" s="4" t="inlineStr"/>
       <c r="H237" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9113,12 +9113,12 @@
         </is>
       </c>
       <c r="F238" s="2" t="n">
-        <v>400.49</v>
+        <v>170.06</v>
       </c>
       <c r="G238" s="2" t="inlineStr"/>
       <c r="H238" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9149,12 +9149,12 @@
         </is>
       </c>
       <c r="F239" s="4" t="n">
-        <v>449.15</v>
+        <v>341.37</v>
       </c>
       <c r="G239" s="4" t="inlineStr"/>
       <c r="H239" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9185,12 +9185,12 @@
         </is>
       </c>
       <c r="F240" s="2" t="n">
-        <v>220.06</v>
+        <v>357.3</v>
       </c>
       <c r="G240" s="2" t="inlineStr"/>
       <c r="H240" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9221,12 +9221,12 @@
         </is>
       </c>
       <c r="F241" s="4" t="n">
-        <v>370.02</v>
+        <v>142.27</v>
       </c>
       <c r="G241" s="4" t="inlineStr"/>
       <c r="H241" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9257,12 +9257,12 @@
         </is>
       </c>
       <c r="F242" s="2" t="n">
-        <v>101.7</v>
+        <v>144</v>
       </c>
       <c r="G242" s="2" t="inlineStr"/>
       <c r="H242" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9293,12 +9293,12 @@
         </is>
       </c>
       <c r="F243" s="4" t="n">
-        <v>258.93</v>
+        <v>270.88</v>
       </c>
       <c r="G243" s="4" t="inlineStr"/>
       <c r="H243" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9329,12 +9329,12 @@
         </is>
       </c>
       <c r="F244" s="2" t="n">
-        <v>239.66</v>
+        <v>348.15</v>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
       <c r="H244" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9365,12 +9365,12 @@
         </is>
       </c>
       <c r="F245" s="4" t="n">
-        <v>210.16</v>
+        <v>419.93</v>
       </c>
       <c r="G245" s="4" t="inlineStr"/>
       <c r="H245" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9401,12 +9401,12 @@
         </is>
       </c>
       <c r="F246" s="2" t="n">
-        <v>331.8</v>
+        <v>163.84</v>
       </c>
       <c r="G246" s="2" t="inlineStr"/>
       <c r="H246" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9437,12 +9437,12 @@
         </is>
       </c>
       <c r="F247" s="4" t="n">
-        <v>295.45</v>
+        <v>283.73</v>
       </c>
       <c r="G247" s="4" t="inlineStr"/>
       <c r="H247" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9473,12 +9473,12 @@
         </is>
       </c>
       <c r="F248" s="2" t="n">
-        <v>243.86</v>
+        <v>422.63</v>
       </c>
       <c r="G248" s="2" t="inlineStr"/>
       <c r="H248" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9509,12 +9509,12 @@
         </is>
       </c>
       <c r="F249" s="4" t="n">
-        <v>139.59</v>
+        <v>86.08</v>
       </c>
       <c r="G249" s="4" t="inlineStr"/>
       <c r="H249" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9545,12 +9545,12 @@
         </is>
       </c>
       <c r="F250" s="2" t="n">
-        <v>197.57</v>
+        <v>371.01</v>
       </c>
       <c r="G250" s="2" t="inlineStr"/>
       <c r="H250" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9581,12 +9581,12 @@
         </is>
       </c>
       <c r="F251" s="4" t="n">
-        <v>61.19</v>
+        <v>336.81</v>
       </c>
       <c r="G251" s="4" t="inlineStr"/>
       <c r="H251" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9617,12 +9617,12 @@
         </is>
       </c>
       <c r="F252" s="2" t="n">
-        <v>61.3</v>
+        <v>361.27</v>
       </c>
       <c r="G252" s="2" t="inlineStr"/>
       <c r="H252" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9653,12 +9653,12 @@
         </is>
       </c>
       <c r="F253" s="4" t="n">
-        <v>161.95</v>
+        <v>90.43000000000001</v>
       </c>
       <c r="G253" s="4" t="inlineStr"/>
       <c r="H253" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9689,12 +9689,12 @@
         </is>
       </c>
       <c r="F254" s="2" t="n">
-        <v>295.62</v>
+        <v>411.23</v>
       </c>
       <c r="G254" s="2" t="inlineStr"/>
       <c r="H254" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9725,12 +9725,12 @@
         </is>
       </c>
       <c r="F255" s="4" t="n">
-        <v>204.96</v>
+        <v>440.06</v>
       </c>
       <c r="G255" s="4" t="inlineStr"/>
       <c r="H255" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9761,12 +9761,12 @@
         </is>
       </c>
       <c r="F256" s="2" t="n">
-        <v>116.9</v>
+        <v>322.02</v>
       </c>
       <c r="G256" s="2" t="inlineStr"/>
       <c r="H256" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9797,12 +9797,12 @@
         </is>
       </c>
       <c r="F257" s="4" t="n">
-        <v>52.07</v>
+        <v>132.8</v>
       </c>
       <c r="G257" s="4" t="inlineStr"/>
       <c r="H257" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9833,12 +9833,12 @@
         </is>
       </c>
       <c r="F258" s="2" t="n">
-        <v>178.14</v>
+        <v>292.54</v>
       </c>
       <c r="G258" s="2" t="inlineStr"/>
       <c r="H258" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9869,12 +9869,12 @@
         </is>
       </c>
       <c r="F259" s="4" t="n">
-        <v>119.51</v>
+        <v>87.43000000000001</v>
       </c>
       <c r="G259" s="4" t="inlineStr"/>
       <c r="H259" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9905,12 +9905,12 @@
         </is>
       </c>
       <c r="F260" s="2" t="n">
-        <v>440.81</v>
+        <v>216.1</v>
       </c>
       <c r="G260" s="2" t="inlineStr"/>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9941,12 +9941,12 @@
         </is>
       </c>
       <c r="F261" s="4" t="n">
-        <v>399.57</v>
+        <v>395.54</v>
       </c>
       <c r="G261" s="4" t="inlineStr"/>
       <c r="H261" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -9977,12 +9977,12 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>209.45</v>
+        <v>235</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
       <c r="H262" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10013,12 +10013,12 @@
         </is>
       </c>
       <c r="F263" s="4" t="n">
-        <v>110.58</v>
+        <v>164.09</v>
       </c>
       <c r="G263" s="4" t="inlineStr"/>
       <c r="H263" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10049,12 +10049,12 @@
         </is>
       </c>
       <c r="F264" s="2" t="n">
-        <v>422.99</v>
+        <v>150.46</v>
       </c>
       <c r="G264" s="2" t="inlineStr"/>
       <c r="H264" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10085,12 +10085,12 @@
         </is>
       </c>
       <c r="F265" s="4" t="n">
-        <v>199.38</v>
+        <v>219.67</v>
       </c>
       <c r="G265" s="4" t="inlineStr"/>
       <c r="H265" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10121,12 +10121,12 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>142.21</v>
+        <v>315.93</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10157,12 +10157,12 @@
         </is>
       </c>
       <c r="F267" s="4" t="n">
-        <v>243.81</v>
+        <v>270.9</v>
       </c>
       <c r="G267" s="4" t="inlineStr"/>
       <c r="H267" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10193,12 +10193,12 @@
         </is>
       </c>
       <c r="F268" s="2" t="n">
-        <v>397.75</v>
+        <v>372.77</v>
       </c>
       <c r="G268" s="2" t="inlineStr"/>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10229,12 +10229,12 @@
         </is>
       </c>
       <c r="F269" s="4" t="n">
-        <v>238.5</v>
+        <v>188.98</v>
       </c>
       <c r="G269" s="4" t="inlineStr"/>
       <c r="H269" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10265,12 +10265,12 @@
         </is>
       </c>
       <c r="F270" s="2" t="n">
-        <v>312.64</v>
+        <v>428.01</v>
       </c>
       <c r="G270" s="2" t="inlineStr"/>
       <c r="H270" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10301,12 +10301,12 @@
         </is>
       </c>
       <c r="F271" s="4" t="n">
-        <v>374.52</v>
+        <v>198.57</v>
       </c>
       <c r="G271" s="4" t="inlineStr"/>
       <c r="H271" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10337,12 +10337,12 @@
         </is>
       </c>
       <c r="F272" s="2" t="n">
-        <v>279.34</v>
+        <v>444.86</v>
       </c>
       <c r="G272" s="2" t="inlineStr"/>
       <c r="H272" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10373,12 +10373,12 @@
         </is>
       </c>
       <c r="F273" s="4" t="n">
-        <v>169.59</v>
+        <v>59.41</v>
       </c>
       <c r="G273" s="4" t="inlineStr"/>
       <c r="H273" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10409,12 +10409,12 @@
         </is>
       </c>
       <c r="F274" s="2" t="n">
-        <v>248.97</v>
+        <v>133.94</v>
       </c>
       <c r="G274" s="2" t="inlineStr"/>
       <c r="H274" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10445,12 +10445,12 @@
         </is>
       </c>
       <c r="F275" s="4" t="n">
-        <v>242.37</v>
+        <v>293.43</v>
       </c>
       <c r="G275" s="4" t="inlineStr"/>
       <c r="H275" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10481,12 +10481,12 @@
         </is>
       </c>
       <c r="F276" s="2" t="n">
-        <v>169.29</v>
+        <v>445.91</v>
       </c>
       <c r="G276" s="2" t="inlineStr"/>
       <c r="H276" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10517,12 +10517,12 @@
         </is>
       </c>
       <c r="F277" s="4" t="n">
-        <v>318</v>
+        <v>163.66</v>
       </c>
       <c r="G277" s="4" t="inlineStr"/>
       <c r="H277" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10553,12 +10553,12 @@
         </is>
       </c>
       <c r="F278" s="2" t="n">
-        <v>395.27</v>
+        <v>405.65</v>
       </c>
       <c r="G278" s="2" t="inlineStr"/>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10589,12 +10589,12 @@
         </is>
       </c>
       <c r="F279" s="4" t="n">
-        <v>203.73</v>
+        <v>190.52</v>
       </c>
       <c r="G279" s="4" t="inlineStr"/>
       <c r="H279" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10625,12 +10625,12 @@
         </is>
       </c>
       <c r="F280" s="2" t="n">
-        <v>167.97</v>
+        <v>300.99</v>
       </c>
       <c r="G280" s="2" t="inlineStr"/>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10661,12 +10661,12 @@
         </is>
       </c>
       <c r="F281" s="4" t="n">
-        <v>317.72</v>
+        <v>74.19</v>
       </c>
       <c r="G281" s="4" t="inlineStr"/>
       <c r="H281" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10697,12 +10697,12 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>109.4</v>
+        <v>240.3</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
       <c r="H282" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10733,12 +10733,12 @@
         </is>
       </c>
       <c r="F283" s="4" t="n">
-        <v>51.75</v>
+        <v>207.55</v>
       </c>
       <c r="G283" s="4" t="inlineStr"/>
       <c r="H283" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10769,12 +10769,12 @@
         </is>
       </c>
       <c r="F284" s="2" t="n">
-        <v>354.4</v>
+        <v>314.82</v>
       </c>
       <c r="G284" s="2" t="inlineStr"/>
       <c r="H284" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10805,12 +10805,12 @@
         </is>
       </c>
       <c r="F285" s="4" t="n">
-        <v>164.87</v>
+        <v>92.48</v>
       </c>
       <c r="G285" s="4" t="inlineStr"/>
       <c r="H285" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10841,12 +10841,12 @@
         </is>
       </c>
       <c r="F286" s="2" t="n">
-        <v>279.63</v>
+        <v>448.92</v>
       </c>
       <c r="G286" s="2" t="inlineStr"/>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10877,12 +10877,12 @@
         </is>
       </c>
       <c r="F287" s="4" t="n">
-        <v>292.97</v>
+        <v>323.3</v>
       </c>
       <c r="G287" s="4" t="inlineStr"/>
       <c r="H287" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10913,12 +10913,12 @@
         </is>
       </c>
       <c r="F288" s="2" t="n">
-        <v>192.87</v>
+        <v>260.24</v>
       </c>
       <c r="G288" s="2" t="inlineStr"/>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10949,12 +10949,12 @@
         </is>
       </c>
       <c r="F289" s="4" t="n">
-        <v>441.41</v>
+        <v>228.02</v>
       </c>
       <c r="G289" s="4" t="inlineStr"/>
       <c r="H289" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -10985,12 +10985,12 @@
         </is>
       </c>
       <c r="F290" s="2" t="n">
-        <v>412.71</v>
+        <v>299.17</v>
       </c>
       <c r="G290" s="2" t="inlineStr"/>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11021,12 +11021,12 @@
         </is>
       </c>
       <c r="F291" s="4" t="n">
-        <v>59.76</v>
+        <v>414.87</v>
       </c>
       <c r="G291" s="4" t="inlineStr"/>
       <c r="H291" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11057,12 +11057,12 @@
         </is>
       </c>
       <c r="F292" s="2" t="n">
-        <v>195.36</v>
+        <v>344.64</v>
       </c>
       <c r="G292" s="2" t="inlineStr"/>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11093,12 +11093,12 @@
         </is>
       </c>
       <c r="F293" s="4" t="n">
-        <v>300.71</v>
+        <v>433.54</v>
       </c>
       <c r="G293" s="4" t="inlineStr"/>
       <c r="H293" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11129,12 +11129,12 @@
         </is>
       </c>
       <c r="F294" s="2" t="n">
-        <v>169.93</v>
+        <v>218.78</v>
       </c>
       <c r="G294" s="2" t="inlineStr"/>
       <c r="H294" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11165,12 +11165,12 @@
         </is>
       </c>
       <c r="F295" s="4" t="n">
-        <v>433.77</v>
+        <v>253.76</v>
       </c>
       <c r="G295" s="4" t="inlineStr"/>
       <c r="H295" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11201,12 +11201,12 @@
         </is>
       </c>
       <c r="F296" s="2" t="n">
-        <v>176.33</v>
+        <v>260.52</v>
       </c>
       <c r="G296" s="2" t="inlineStr"/>
       <c r="H296" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11237,12 +11237,12 @@
         </is>
       </c>
       <c r="F297" s="4" t="n">
-        <v>98.31</v>
+        <v>183.71</v>
       </c>
       <c r="G297" s="4" t="inlineStr"/>
       <c r="H297" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11273,12 +11273,12 @@
         </is>
       </c>
       <c r="F298" s="2" t="n">
-        <v>99.42</v>
+        <v>228.3</v>
       </c>
       <c r="G298" s="2" t="inlineStr"/>
       <c r="H298" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11309,12 +11309,12 @@
         </is>
       </c>
       <c r="F299" s="4" t="n">
-        <v>148.23</v>
+        <v>230.72</v>
       </c>
       <c r="G299" s="4" t="inlineStr"/>
       <c r="H299" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11345,12 +11345,12 @@
         </is>
       </c>
       <c r="F300" s="2" t="n">
-        <v>420.44</v>
+        <v>74.95</v>
       </c>
       <c r="G300" s="2" t="inlineStr"/>
       <c r="H300" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11381,12 +11381,12 @@
         </is>
       </c>
       <c r="F301" s="4" t="n">
-        <v>198.5</v>
+        <v>295.47</v>
       </c>
       <c r="G301" s="4" t="inlineStr"/>
       <c r="H301" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:38:37</t>
+          <t>2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>
@@ -11418,7 +11418,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Generated: 2026-08-01 09:38:38</t>
+          <t>Generated: 2026-08-01 13:36:49</t>
         </is>
       </c>
     </row>

</xml_diff>